<commit_message>
updated runs for BOOST (longer). Added support for different binaries
</commit_message>
<xml_diff>
--- a/gemini8048/bin/klr_memory_map.xlsx
+++ b/gemini8048/bin/klr_memory_map.xlsx
@@ -663,11 +663,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B27"/>
+  <dimension ref="A1:C27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="75" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="65" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -685,6 +686,11 @@
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
+          <t>Variable Name</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
           <t>Purpose</t>
         </is>
       </c>
@@ -695,7 +701,12 @@
           <t>24h</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>ENGINE_SPEED_COMPLEMENT</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
         <is>
           <t>engine speed (complemented from r6; literally 87us timer ticks per 180 degrees)</t>
         </is>
@@ -707,7 +718,12 @@
           <t>2Eh</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>BATTERY_VOLTAGE</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
         <is>
           <t>battery voltage</t>
         </is>
@@ -719,7 +735,12 @@
           <t>2Fh</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>KNOCK_SENSOR_DIAG</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
         <is>
           <t>knock sensor (diagnostics)</t>
         </is>
@@ -731,7 +752,12 @@
           <t>39h</t>
         </is>
       </c>
-      <c r="B7" s="9" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>TPS_POWER_SUPPLY</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
         <is>
           <t>throttle position (power supply)</t>
         </is>
@@ -743,7 +769,12 @@
           <t>3Ah</t>
         </is>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>TPS_DEGREES</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
         <is>
           <t>throttle position (degrees)</t>
         </is>
@@ -755,7 +786,12 @@
           <t>3Ch</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>TPS_RAW</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
         <is>
           <t>throttle position (raw)</t>
         </is>
@@ -767,7 +803,12 @@
           <t>3Fh</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>UNKNOWN_3F</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
         <is>
           <t>??</t>
         </is>
@@ -779,7 +820,12 @@
           <t>38h</t>
         </is>
       </c>
-      <c r="B11" s="9" t="inlineStr">
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>UNKNOWN_38</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
         <is>
           <t>??</t>
         </is>
@@ -791,7 +837,12 @@
           <t>46h</t>
         </is>
       </c>
-      <c r="B12" s="9" t="inlineStr">
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>KNOCK_SENSOR</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
         <is>
           <t>knock sensor (proper)</t>
         </is>
@@ -803,7 +854,12 @@
           <t>24h</t>
         </is>
       </c>
-      <c r="B13" s="9" t="inlineStr">
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>ENGINE_SPEED_TICKS</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
         <is>
           <t>engine speed (in timer ticks)</t>
         </is>
@@ -815,7 +871,12 @@
           <t>52h</t>
         </is>
       </c>
-      <c r="B14" s="9" t="inlineStr">
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>MAP_PRESSURE</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
         <is>
           <t>MAP pressure</t>
         </is>
@@ -827,7 +888,12 @@
           <t>33h</t>
         </is>
       </c>
-      <c r="B15" s="9" t="inlineStr">
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>BLINK_CODE_CURRENT</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
         <is>
           <t>current blink code</t>
         </is>
@@ -839,7 +905,12 @@
           <t>22h</t>
         </is>
       </c>
-      <c r="B16" s="9" t="inlineStr">
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>ADC_INIT_ANGLE</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
         <is>
           <t>angle to begin ADC initialization routine (in timer ticks)</t>
         </is>
@@ -851,7 +922,12 @@
           <t>23h</t>
         </is>
       </c>
-      <c r="B17" s="9" t="inlineStr">
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>ADC_READ_ANGLE</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
         <is>
           <t>angle to read ADC (after 22h, in timer ticks)</t>
         </is>
@@ -863,7 +939,12 @@
           <t>44h</t>
         </is>
       </c>
-      <c r="B18" s="9" t="inlineStr">
+      <c r="B18" s="8" t="inlineStr">
+        <is>
+          <t>RPM_MAP_AXIS</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
         <is>
           <t>rpm range (map axis)</t>
         </is>
@@ -875,7 +956,12 @@
           <t>43h</t>
         </is>
       </c>
-      <c r="B19" s="9" t="inlineStr">
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>TPS_MAP_AXIS</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="inlineStr">
         <is>
           <t>throttle position (map axis)</t>
         </is>
@@ -887,7 +973,12 @@
           <t>70h - 73h</t>
         </is>
       </c>
-      <c r="B20" s="9" t="inlineStr">
+      <c r="B20" s="8" t="inlineStr">
+        <is>
+          <t>CYL_TIMING_DELAY</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="inlineStr">
         <is>
           <t>per-cylinder timing delay</t>
         </is>
@@ -899,7 +990,12 @@
           <t>74h - 7Bh</t>
         </is>
       </c>
-      <c r="B21" s="9" t="inlineStr">
+      <c r="B21" s="8" t="inlineStr">
+        <is>
+          <t>CYL_KNOCK_THRESH</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="inlineStr">
         <is>
           <t>per-cylinder knock threshold</t>
         </is>
@@ -911,7 +1007,12 @@
           <t>60h</t>
         </is>
       </c>
-      <c r="B22" s="9" t="inlineStr">
+      <c r="B22" s="8" t="inlineStr">
+        <is>
+          <t>BOOST_PID_ERROR</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
         <is>
           <t>boost control PID error (target boost - actual boost)</t>
         </is>
@@ -923,7 +1024,12 @@
           <t>61h</t>
         </is>
       </c>
-      <c r="B23" s="9" t="inlineStr">
+      <c r="B23" s="8" t="inlineStr">
+        <is>
+          <t>BOOST_PID_ITERM</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="inlineStr">
         <is>
           <t>boost control PID I term (integral)</t>
         </is>
@@ -935,7 +1041,12 @@
           <t>62h</t>
         </is>
       </c>
-      <c r="B24" s="9" t="inlineStr">
+      <c r="B24" s="8" t="inlineStr">
+        <is>
+          <t>BOOST_PID_DTERM</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="inlineStr">
         <is>
           <t>boost control PID D term (derivative)</t>
         </is>
@@ -947,7 +1058,12 @@
           <t>68h</t>
         </is>
       </c>
-      <c r="B25" s="9" t="inlineStr">
+      <c r="B25" s="8" t="inlineStr">
+        <is>
+          <t>BOOST_FEEDFORWARD_CV</t>
+        </is>
+      </c>
+      <c r="C25" s="9" t="inlineStr">
         <is>
           <t>boost control feedforward value (CV duty cycle)</t>
         </is>
@@ -959,7 +1075,12 @@
           <t>41h</t>
         </is>
       </c>
-      <c r="B26" s="9" t="inlineStr">
+      <c r="B26" s="8" t="inlineStr">
+        <is>
+          <t>CV_DUTY_FINAL</t>
+        </is>
+      </c>
+      <c r="C26" s="9" t="inlineStr">
         <is>
           <t>final CV duty cycle</t>
         </is>
@@ -971,7 +1092,12 @@
           <t>57h</t>
         </is>
       </c>
-      <c r="B27" s="9" t="inlineStr">
+      <c r="B27" s="8" t="inlineStr">
+        <is>
+          <t>BOOST_REDUCTION_KNOCK</t>
+        </is>
+      </c>
+      <c r="C27" s="9" t="inlineStr">
         <is>
           <t>total boost reduction for knock control</t>
         </is>
@@ -988,11 +1114,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1010,6 +1137,11 @@
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
+          <t>Variable Name</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
           <t>Error Type</t>
         </is>
       </c>
@@ -1020,7 +1152,12 @@
           <t>30h</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>BLINK_ERR_KNOCK_MAP</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
         <is>
           <t>knock/MAP</t>
         </is>
@@ -1032,7 +1169,12 @@
           <t>35h</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>BLINK_ERR_BOOST_HILO</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
         <is>
           <t>boost high/low</t>
         </is>
@@ -1044,7 +1186,12 @@
           <t>36h</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>BLINK_ERR_TPS</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
         <is>
           <t>TPS/TPS power supply</t>
         </is>
@@ -1061,11 +1208,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="55" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1090,6 +1238,11 @@
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
+          <t>Variable Name</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
           <t>Purpose</t>
         </is>
       </c>
@@ -1100,7 +1253,12 @@
           <t>0x2A</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>RPM_K_ADC_START_ANGLE</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
         <is>
           <t>for calculating the angle to start ADC stuff (22h)</t>
         </is>
@@ -1112,7 +1270,12 @@
           <t>0x2B</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>RPM_K_ADC_READ_ANGLE</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
         <is>
           <t>for calculating the angle for ADC read (23h)</t>
         </is>
@@ -1124,7 +1287,12 @@
           <t>0x47</t>
         </is>
       </c>
-      <c r="B7" s="9" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>RPM_K_KNOCK_THRESH_COEF</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
         <is>
           <t>coefficient for knock threshold (comparison with 46h)</t>
         </is>
@@ -1136,7 +1304,12 @@
           <t>0x4A</t>
         </is>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>RPM_K_TIMING_RESTORE_CNT</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
         <is>
           <t>cycle count before restoring 0.3 deg. timing (49h)</t>
         </is>
@@ -1148,7 +1321,12 @@
           <t>0x50</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>RPM_K_BOOST_RESTORE_CNT</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
         <is>
           <t>cycle count before restoring boost (15 to 37)</t>
         </is>
@@ -1160,7 +1338,12 @@
           <t>0x4E</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>RPM_K_BOOST_PULL_CNT</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
         <is>
           <t>cycle count before pulling boost (31 to 125)</t>
         </is>
@@ -1172,7 +1355,12 @@
           <t>0x4B</t>
         </is>
       </c>
-      <c r="B11" s="9" t="inlineStr">
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>RPM_K_MAX_TIMING_RETARD</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
         <is>
           <t>max timing retard (18 dec. for all rpm)</t>
         </is>
@@ -1184,7 +1372,12 @@
           <t>0x48</t>
         </is>
       </c>
-      <c r="B12" s="9" t="inlineStr">
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>RPM_K_KNOCK_TPS_THRESH</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
         <is>
           <t>throttle position threshhold for knock control</t>
         </is>
@@ -1196,7 +1389,12 @@
           <t>0x4C</t>
         </is>
       </c>
-      <c r="B13" s="9" t="inlineStr">
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>RPM_K_BOOST_PULL_THRESH</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
         <is>
           <t>threshold for pulling boost</t>
         </is>
@@ -1208,7 +1406,12 @@
           <t>0x3E</t>
         </is>
       </c>
-      <c r="B14" s="9" t="inlineStr">
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>RPM_K_WOT_ANGLE</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
         <is>
           <t>angle for WOT (set to 66 decimal for all rpm)</t>
         </is>
@@ -1220,7 +1423,12 @@
           <t>0x45</t>
         </is>
       </c>
-      <c r="B15" s="9" t="inlineStr">
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>RPM_K_MIN_KNOCK_THRESH</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
         <is>
           <t>minimum knock threshold value (10 for all rpm)</t>
         </is>
@@ -1232,7 +1440,12 @@
           <t>0x69</t>
         </is>
       </c>
-      <c r="B16" s="9" t="inlineStr">
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>RPM_K_CNT_FOR_6A</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
         <is>
           <t>counter for 6A (set to 4 for all rpm)</t>
         </is>

</xml_diff>